<commit_message>
Update renewable generator dashboard data 2026-05
</commit_message>
<xml_diff>
--- a/outputs/SA_curtailment.xlsx
+++ b/outputs/SA_curtailment.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Heatmap" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -67,7 +67,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" wrapText="1"/>
@@ -82,9 +82,6 @@
       <alignment horizontal="right"/>
     </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -456,7 +453,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:W47"/>
+  <dimension ref="A1:O47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -474,14 +471,6 @@
     <col width="12" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="12" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="12" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
-    <col width="12" customWidth="1" min="19" max="19"/>
-    <col width="12" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
-    <col width="12" customWidth="1" min="22" max="22"/>
-    <col width="12" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -560,46 +549,6 @@
           <t>FY26-27</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
-        <is>
-          <t>Curt FY1</t>
-        </is>
-      </c>
-      <c r="Q1" s="1" t="inlineStr">
-        <is>
-          <t>Curt FY2</t>
-        </is>
-      </c>
-      <c r="R1" s="1" t="inlineStr">
-        <is>
-          <t>Curt FY3</t>
-        </is>
-      </c>
-      <c r="S1" s="1" t="inlineStr">
-        <is>
-          <t>Curt Avg</t>
-        </is>
-      </c>
-      <c r="T1" s="1" t="inlineStr">
-        <is>
-          <t>Offl FY1</t>
-        </is>
-      </c>
-      <c r="U1" s="1" t="inlineStr">
-        <is>
-          <t>Offl FY2</t>
-        </is>
-      </c>
-      <c r="V1" s="1" t="inlineStr">
-        <is>
-          <t>Offl FY3</t>
-        </is>
-      </c>
-      <c r="W1" s="1" t="inlineStr">
-        <is>
-          <t>Offl Avg</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -651,14 +600,6 @@
       <c r="O2" s="5" t="n">
         <v>1.0033</v>
       </c>
-      <c r="P2" s="6" t="inlineStr"/>
-      <c r="Q2" s="6" t="inlineStr"/>
-      <c r="R2" s="6" t="inlineStr"/>
-      <c r="S2" s="6" t="inlineStr"/>
-      <c r="T2" s="6" t="inlineStr"/>
-      <c r="U2" s="6" t="inlineStr"/>
-      <c r="V2" s="6" t="inlineStr"/>
-      <c r="W2" s="6" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -706,14 +647,6 @@
       <c r="O3" s="5" t="n">
         <v>1.0033</v>
       </c>
-      <c r="P3" s="6" t="inlineStr"/>
-      <c r="Q3" s="6" t="inlineStr"/>
-      <c r="R3" s="6" t="inlineStr"/>
-      <c r="S3" s="6" t="inlineStr"/>
-      <c r="T3" s="6" t="inlineStr"/>
-      <c r="U3" s="6" t="inlineStr"/>
-      <c r="V3" s="6" t="inlineStr"/>
-      <c r="W3" s="6" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -761,14 +694,6 @@
       <c r="O4" s="5" t="n">
         <v>1.0033</v>
       </c>
-      <c r="P4" s="6" t="inlineStr"/>
-      <c r="Q4" s="6" t="inlineStr"/>
-      <c r="R4" s="6" t="inlineStr"/>
-      <c r="S4" s="6" t="inlineStr"/>
-      <c r="T4" s="6" t="inlineStr"/>
-      <c r="U4" s="6" t="inlineStr"/>
-      <c r="V4" s="6" t="inlineStr"/>
-      <c r="W4" s="6" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -818,14 +743,6 @@
       <c r="O5" s="5" t="n">
         <v>1.0002</v>
       </c>
-      <c r="P5" s="6" t="inlineStr"/>
-      <c r="Q5" s="6" t="inlineStr"/>
-      <c r="R5" s="6" t="inlineStr"/>
-      <c r="S5" s="6" t="inlineStr"/>
-      <c r="T5" s="6" t="inlineStr"/>
-      <c r="U5" s="6" t="inlineStr"/>
-      <c r="V5" s="6" t="inlineStr"/>
-      <c r="W5" s="6" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -887,30 +804,6 @@
       <c r="O6" s="5" t="n">
         <v>0.9703000000000001</v>
       </c>
-      <c r="P6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S6" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T6" s="6" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="U6" s="6" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="V6" s="6" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="W6" s="6" t="n">
-        <v>0.07333333333333335</v>
-      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -971,30 +864,6 @@
       </c>
       <c r="O7" s="5" t="n">
         <v>0.9703000000000001</v>
-      </c>
-      <c r="P7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S7" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T7" s="6" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="U7" s="6" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="V7" s="6" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="W7" s="6" t="n">
-        <v>0.07333333333333335</v>
       </c>
     </row>
     <row r="8">
@@ -1043,14 +912,6 @@
       <c r="O8" s="5" t="n">
         <v>1.0033</v>
       </c>
-      <c r="P8" s="6" t="inlineStr"/>
-      <c r="Q8" s="6" t="inlineStr"/>
-      <c r="R8" s="6" t="inlineStr"/>
-      <c r="S8" s="6" t="inlineStr"/>
-      <c r="T8" s="6" t="inlineStr"/>
-      <c r="U8" s="6" t="inlineStr"/>
-      <c r="V8" s="6" t="inlineStr"/>
-      <c r="W8" s="6" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -1098,14 +959,6 @@
       <c r="O9" s="5" t="n">
         <v>1.0033</v>
       </c>
-      <c r="P9" s="6" t="inlineStr"/>
-      <c r="Q9" s="6" t="inlineStr"/>
-      <c r="R9" s="6" t="inlineStr"/>
-      <c r="S9" s="6" t="inlineStr"/>
-      <c r="T9" s="6" t="inlineStr"/>
-      <c r="U9" s="6" t="inlineStr"/>
-      <c r="V9" s="6" t="inlineStr"/>
-      <c r="W9" s="6" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -1167,14 +1020,6 @@
       <c r="O10" s="5" t="n">
         <v>1.0022</v>
       </c>
-      <c r="P10" s="6" t="inlineStr"/>
-      <c r="Q10" s="6" t="inlineStr"/>
-      <c r="R10" s="6" t="inlineStr"/>
-      <c r="S10" s="6" t="inlineStr"/>
-      <c r="T10" s="6" t="inlineStr"/>
-      <c r="U10" s="6" t="inlineStr"/>
-      <c r="V10" s="6" t="inlineStr"/>
-      <c r="W10" s="6" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -1235,30 +1080,6 @@
       </c>
       <c r="O11" s="5" t="n">
         <v>1.0134</v>
-      </c>
-      <c r="P11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V11" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W11" s="6" t="n">
-        <v>0</v>
       </c>
     </row>
     <row r="12">
@@ -1319,30 +1140,6 @@
       <c r="O12" s="5" t="n">
         <v>1.0137</v>
       </c>
-      <c r="P12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V12" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W12" s="6" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -1402,30 +1199,6 @@
       <c r="O13" s="5" t="n">
         <v>0.9959</v>
       </c>
-      <c r="P13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S13" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T13" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U13" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="V13" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="W13" s="6" t="n">
-        <v>0.16</v>
-      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -1487,30 +1260,6 @@
       <c r="O14" s="5" t="n">
         <v>0.9540999999999999</v>
       </c>
-      <c r="P14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S14" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T14" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U14" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="V14" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="W14" s="6" t="n">
-        <v>0.16</v>
-      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -1572,30 +1321,6 @@
       <c r="O15" s="5" t="n">
         <v>0.9664</v>
       </c>
-      <c r="P15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S15" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T15" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U15" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="V15" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="W15" s="6" t="n">
-        <v>0.16</v>
-      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -1657,30 +1382,6 @@
       <c r="O16" s="5" t="n">
         <v>0.9741</v>
       </c>
-      <c r="P16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S16" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T16" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U16" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="V16" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="W16" s="6" t="n">
-        <v>0.16</v>
-      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -1742,30 +1443,6 @@
       <c r="O17" s="5" t="n">
         <v>0.9772999999999999</v>
       </c>
-      <c r="P17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S17" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T17" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U17" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="V17" s="6" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="W17" s="6" t="n">
-        <v>0.16</v>
-      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -1827,30 +1504,6 @@
       <c r="O18" s="5" t="n">
         <v>1.011</v>
       </c>
-      <c r="P18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="U18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="V18" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="W18" s="6" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -1912,30 +1565,6 @@
       <c r="O19" s="5" t="n">
         <v>0.9709</v>
       </c>
-      <c r="P19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="R19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="S19" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="T19" s="6" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="U19" s="6" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="V19" s="6" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="W19" s="6" t="n">
-        <v>0.07333333333333335</v>
-      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -1997,14 +1626,6 @@
       <c r="O20" s="5" t="n">
         <v>0.9968</v>
       </c>
-      <c r="P20" s="6" t="inlineStr"/>
-      <c r="Q20" s="6" t="inlineStr"/>
-      <c r="R20" s="6" t="inlineStr"/>
-      <c r="S20" s="6" t="inlineStr"/>
-      <c r="T20" s="6" t="inlineStr"/>
-      <c r="U20" s="6" t="inlineStr"/>
-      <c r="V20" s="6" t="inlineStr"/>
-      <c r="W20" s="6" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -2066,14 +1687,6 @@
       <c r="O21" s="5" t="n">
         <v>0.9978</v>
       </c>
-      <c r="P21" s="6" t="inlineStr"/>
-      <c r="Q21" s="6" t="inlineStr"/>
-      <c r="R21" s="6" t="inlineStr"/>
-      <c r="S21" s="6" t="inlineStr"/>
-      <c r="T21" s="6" t="inlineStr"/>
-      <c r="U21" s="6" t="inlineStr"/>
-      <c r="V21" s="6" t="inlineStr"/>
-      <c r="W21" s="6" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -2125,14 +1738,6 @@
       <c r="O22" s="5" t="n">
         <v>0.9527</v>
       </c>
-      <c r="P22" s="6" t="inlineStr"/>
-      <c r="Q22" s="6" t="inlineStr"/>
-      <c r="R22" s="6" t="inlineStr"/>
-      <c r="S22" s="6" t="inlineStr"/>
-      <c r="T22" s="6" t="inlineStr"/>
-      <c r="U22" s="6" t="inlineStr"/>
-      <c r="V22" s="6" t="inlineStr"/>
-      <c r="W22" s="6" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -2184,14 +1789,6 @@
       <c r="O23" s="5" t="n">
         <v>0.9417</v>
       </c>
-      <c r="P23" s="6" t="inlineStr"/>
-      <c r="Q23" s="6" t="inlineStr"/>
-      <c r="R23" s="6" t="inlineStr"/>
-      <c r="S23" s="6" t="inlineStr"/>
-      <c r="T23" s="6" t="inlineStr"/>
-      <c r="U23" s="6" t="inlineStr"/>
-      <c r="V23" s="6" t="inlineStr"/>
-      <c r="W23" s="6" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -2243,14 +1840,6 @@
       <c r="O24" s="5" t="n">
         <v>0.9614</v>
       </c>
-      <c r="P24" s="6" t="inlineStr"/>
-      <c r="Q24" s="6" t="inlineStr"/>
-      <c r="R24" s="6" t="inlineStr"/>
-      <c r="S24" s="6" t="inlineStr"/>
-      <c r="T24" s="6" t="inlineStr"/>
-      <c r="U24" s="6" t="inlineStr"/>
-      <c r="V24" s="6" t="inlineStr"/>
-      <c r="W24" s="6" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -2300,14 +1889,6 @@
       <c r="O25" s="5" t="n">
         <v>0.9687</v>
       </c>
-      <c r="P25" s="6" t="inlineStr"/>
-      <c r="Q25" s="6" t="inlineStr"/>
-      <c r="R25" s="6" t="inlineStr"/>
-      <c r="S25" s="6" t="inlineStr"/>
-      <c r="T25" s="6" t="inlineStr"/>
-      <c r="U25" s="6" t="inlineStr"/>
-      <c r="V25" s="6" t="inlineStr"/>
-      <c r="W25" s="6" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -2355,14 +1936,6 @@
       <c r="O26" s="5" t="n">
         <v>0.9687</v>
       </c>
-      <c r="P26" s="6" t="inlineStr"/>
-      <c r="Q26" s="6" t="inlineStr"/>
-      <c r="R26" s="6" t="inlineStr"/>
-      <c r="S26" s="6" t="inlineStr"/>
-      <c r="T26" s="6" t="inlineStr"/>
-      <c r="U26" s="6" t="inlineStr"/>
-      <c r="V26" s="6" t="inlineStr"/>
-      <c r="W26" s="6" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -2414,14 +1987,6 @@
       <c r="O27" s="5" t="n">
         <v>0.9628</v>
       </c>
-      <c r="P27" s="6" t="inlineStr"/>
-      <c r="Q27" s="6" t="inlineStr"/>
-      <c r="R27" s="6" t="inlineStr"/>
-      <c r="S27" s="6" t="inlineStr"/>
-      <c r="T27" s="6" t="inlineStr"/>
-      <c r="U27" s="6" t="inlineStr"/>
-      <c r="V27" s="6" t="inlineStr"/>
-      <c r="W27" s="6" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -2473,14 +2038,6 @@
       <c r="O28" s="5" t="n">
         <v>0.9606</v>
       </c>
-      <c r="P28" s="6" t="inlineStr"/>
-      <c r="Q28" s="6" t="inlineStr"/>
-      <c r="R28" s="6" t="inlineStr"/>
-      <c r="S28" s="6" t="inlineStr"/>
-      <c r="T28" s="6" t="inlineStr"/>
-      <c r="U28" s="6" t="inlineStr"/>
-      <c r="V28" s="6" t="inlineStr"/>
-      <c r="W28" s="6" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -2532,14 +2089,6 @@
       <c r="O29" s="5" t="n">
         <v>0.9533</v>
       </c>
-      <c r="P29" s="6" t="inlineStr"/>
-      <c r="Q29" s="6" t="inlineStr"/>
-      <c r="R29" s="6" t="inlineStr"/>
-      <c r="S29" s="6" t="inlineStr"/>
-      <c r="T29" s="6" t="inlineStr"/>
-      <c r="U29" s="6" t="inlineStr"/>
-      <c r="V29" s="6" t="inlineStr"/>
-      <c r="W29" s="6" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -2591,14 +2140,6 @@
       <c r="O30" s="5" t="n">
         <v>0.9533</v>
       </c>
-      <c r="P30" s="6" t="inlineStr"/>
-      <c r="Q30" s="6" t="inlineStr"/>
-      <c r="R30" s="6" t="inlineStr"/>
-      <c r="S30" s="6" t="inlineStr"/>
-      <c r="T30" s="6" t="inlineStr"/>
-      <c r="U30" s="6" t="inlineStr"/>
-      <c r="V30" s="6" t="inlineStr"/>
-      <c r="W30" s="6" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -2650,14 +2191,6 @@
       <c r="O31" s="5" t="n">
         <v>0.9533</v>
       </c>
-      <c r="P31" s="6" t="inlineStr"/>
-      <c r="Q31" s="6" t="inlineStr"/>
-      <c r="R31" s="6" t="inlineStr"/>
-      <c r="S31" s="6" t="inlineStr"/>
-      <c r="T31" s="6" t="inlineStr"/>
-      <c r="U31" s="6" t="inlineStr"/>
-      <c r="V31" s="6" t="inlineStr"/>
-      <c r="W31" s="6" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -2709,14 +2242,6 @@
       <c r="O32" s="5" t="n">
         <v>0.9468</v>
       </c>
-      <c r="P32" s="6" t="inlineStr"/>
-      <c r="Q32" s="6" t="inlineStr"/>
-      <c r="R32" s="6" t="inlineStr"/>
-      <c r="S32" s="6" t="inlineStr"/>
-      <c r="T32" s="6" t="inlineStr"/>
-      <c r="U32" s="6" t="inlineStr"/>
-      <c r="V32" s="6" t="inlineStr"/>
-      <c r="W32" s="6" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -2768,14 +2293,6 @@
       <c r="O33" s="5" t="n">
         <v>0.9468</v>
       </c>
-      <c r="P33" s="6" t="inlineStr"/>
-      <c r="Q33" s="6" t="inlineStr"/>
-      <c r="R33" s="6" t="inlineStr"/>
-      <c r="S33" s="6" t="inlineStr"/>
-      <c r="T33" s="6" t="inlineStr"/>
-      <c r="U33" s="6" t="inlineStr"/>
-      <c r="V33" s="6" t="inlineStr"/>
-      <c r="W33" s="6" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -2827,14 +2344,6 @@
       <c r="O34" s="5" t="n">
         <v>0.9468</v>
       </c>
-      <c r="P34" s="6" t="inlineStr"/>
-      <c r="Q34" s="6" t="inlineStr"/>
-      <c r="R34" s="6" t="inlineStr"/>
-      <c r="S34" s="6" t="inlineStr"/>
-      <c r="T34" s="6" t="inlineStr"/>
-      <c r="U34" s="6" t="inlineStr"/>
-      <c r="V34" s="6" t="inlineStr"/>
-      <c r="W34" s="6" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -2886,14 +2395,6 @@
       <c r="O35" s="5" t="n">
         <v>0.9661</v>
       </c>
-      <c r="P35" s="6" t="inlineStr"/>
-      <c r="Q35" s="6" t="inlineStr"/>
-      <c r="R35" s="6" t="inlineStr"/>
-      <c r="S35" s="6" t="inlineStr"/>
-      <c r="T35" s="6" t="inlineStr"/>
-      <c r="U35" s="6" t="inlineStr"/>
-      <c r="V35" s="6" t="inlineStr"/>
-      <c r="W35" s="6" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" s="2" t="inlineStr">
@@ -2945,14 +2446,6 @@
       <c r="O36" s="5" t="n">
         <v>0.9661</v>
       </c>
-      <c r="P36" s="6" t="inlineStr"/>
-      <c r="Q36" s="6" t="inlineStr"/>
-      <c r="R36" s="6" t="inlineStr"/>
-      <c r="S36" s="6" t="inlineStr"/>
-      <c r="T36" s="6" t="inlineStr"/>
-      <c r="U36" s="6" t="inlineStr"/>
-      <c r="V36" s="6" t="inlineStr"/>
-      <c r="W36" s="6" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -3004,14 +2497,6 @@
       <c r="O37" s="5" t="n">
         <v>0.9387</v>
       </c>
-      <c r="P37" s="6" t="inlineStr"/>
-      <c r="Q37" s="6" t="inlineStr"/>
-      <c r="R37" s="6" t="inlineStr"/>
-      <c r="S37" s="6" t="inlineStr"/>
-      <c r="T37" s="6" t="inlineStr"/>
-      <c r="U37" s="6" t="inlineStr"/>
-      <c r="V37" s="6" t="inlineStr"/>
-      <c r="W37" s="6" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -3063,14 +2548,6 @@
       <c r="O38" s="5" t="n">
         <v>0.9572000000000001</v>
       </c>
-      <c r="P38" s="6" t="inlineStr"/>
-      <c r="Q38" s="6" t="inlineStr"/>
-      <c r="R38" s="6" t="inlineStr"/>
-      <c r="S38" s="6" t="inlineStr"/>
-      <c r="T38" s="6" t="inlineStr"/>
-      <c r="U38" s="6" t="inlineStr"/>
-      <c r="V38" s="6" t="inlineStr"/>
-      <c r="W38" s="6" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -3122,14 +2599,6 @@
       <c r="O39" s="5" t="n">
         <v>0.9709</v>
       </c>
-      <c r="P39" s="6" t="inlineStr"/>
-      <c r="Q39" s="6" t="inlineStr"/>
-      <c r="R39" s="6" t="inlineStr"/>
-      <c r="S39" s="6" t="inlineStr"/>
-      <c r="T39" s="6" t="inlineStr"/>
-      <c r="U39" s="6" t="inlineStr"/>
-      <c r="V39" s="6" t="inlineStr"/>
-      <c r="W39" s="6" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -3181,14 +2650,6 @@
       <c r="O40" s="5" t="n">
         <v>0.9699</v>
       </c>
-      <c r="P40" s="6" t="inlineStr"/>
-      <c r="Q40" s="6" t="inlineStr"/>
-      <c r="R40" s="6" t="inlineStr"/>
-      <c r="S40" s="6" t="inlineStr"/>
-      <c r="T40" s="6" t="inlineStr"/>
-      <c r="U40" s="6" t="inlineStr"/>
-      <c r="V40" s="6" t="inlineStr"/>
-      <c r="W40" s="6" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -3240,14 +2701,6 @@
       <c r="O41" s="5" t="n">
         <v>0.9699</v>
       </c>
-      <c r="P41" s="6" t="inlineStr"/>
-      <c r="Q41" s="6" t="inlineStr"/>
-      <c r="R41" s="6" t="inlineStr"/>
-      <c r="S41" s="6" t="inlineStr"/>
-      <c r="T41" s="6" t="inlineStr"/>
-      <c r="U41" s="6" t="inlineStr"/>
-      <c r="V41" s="6" t="inlineStr"/>
-      <c r="W41" s="6" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -3299,14 +2752,6 @@
       <c r="O42" s="5" t="n">
         <v>0.9132</v>
       </c>
-      <c r="P42" s="6" t="inlineStr"/>
-      <c r="Q42" s="6" t="inlineStr"/>
-      <c r="R42" s="6" t="inlineStr"/>
-      <c r="S42" s="6" t="inlineStr"/>
-      <c r="T42" s="6" t="inlineStr"/>
-      <c r="U42" s="6" t="inlineStr"/>
-      <c r="V42" s="6" t="inlineStr"/>
-      <c r="W42" s="6" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -3358,14 +2803,6 @@
       <c r="O43" s="5" t="n">
         <v>1.0033</v>
       </c>
-      <c r="P43" s="6" t="inlineStr"/>
-      <c r="Q43" s="6" t="inlineStr"/>
-      <c r="R43" s="6" t="inlineStr"/>
-      <c r="S43" s="6" t="inlineStr"/>
-      <c r="T43" s="6" t="inlineStr"/>
-      <c r="U43" s="6" t="inlineStr"/>
-      <c r="V43" s="6" t="inlineStr"/>
-      <c r="W43" s="6" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -3417,14 +2854,6 @@
       <c r="O44" s="5" t="n">
         <v>0.9572000000000001</v>
       </c>
-      <c r="P44" s="6" t="inlineStr"/>
-      <c r="Q44" s="6" t="inlineStr"/>
-      <c r="R44" s="6" t="inlineStr"/>
-      <c r="S44" s="6" t="inlineStr"/>
-      <c r="T44" s="6" t="inlineStr"/>
-      <c r="U44" s="6" t="inlineStr"/>
-      <c r="V44" s="6" t="inlineStr"/>
-      <c r="W44" s="6" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -3476,14 +2905,6 @@
       <c r="O45" s="5" t="n">
         <v>0.9611</v>
       </c>
-      <c r="P45" s="6" t="inlineStr"/>
-      <c r="Q45" s="6" t="inlineStr"/>
-      <c r="R45" s="6" t="inlineStr"/>
-      <c r="S45" s="6" t="inlineStr"/>
-      <c r="T45" s="6" t="inlineStr"/>
-      <c r="U45" s="6" t="inlineStr"/>
-      <c r="V45" s="6" t="inlineStr"/>
-      <c r="W45" s="6" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -3535,14 +2956,6 @@
       <c r="O46" s="5" t="n">
         <v>0.8476</v>
       </c>
-      <c r="P46" s="6" t="inlineStr"/>
-      <c r="Q46" s="6" t="inlineStr"/>
-      <c r="R46" s="6" t="inlineStr"/>
-      <c r="S46" s="6" t="inlineStr"/>
-      <c r="T46" s="6" t="inlineStr"/>
-      <c r="U46" s="6" t="inlineStr"/>
-      <c r="V46" s="6" t="inlineStr"/>
-      <c r="W46" s="6" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -3594,14 +3007,6 @@
       <c r="O47" s="5" t="n">
         <v>0.9592000000000001</v>
       </c>
-      <c r="P47" s="6" t="inlineStr"/>
-      <c r="Q47" s="6" t="inlineStr"/>
-      <c r="R47" s="6" t="inlineStr"/>
-      <c r="S47" s="6" t="inlineStr"/>
-      <c r="T47" s="6" t="inlineStr"/>
-      <c r="U47" s="6" t="inlineStr"/>
-      <c r="V47" s="6" t="inlineStr"/>
-      <c r="W47" s="6" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -3614,7 +3019,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:V47"/>
+  <dimension ref="A1:H47"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -3625,141 +3030,57 @@
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="14" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
-    <col width="14" customWidth="1" min="16" max="16"/>
-    <col width="14" customWidth="1" min="17" max="17"/>
-    <col width="14" customWidth="1" min="18" max="18"/>
-    <col width="14" customWidth="1" min="19" max="19"/>
-    <col width="14" customWidth="1" min="20" max="20"/>
-    <col width="14" customWidth="1" min="21" max="21"/>
-    <col width="14" customWidth="1" min="22" max="22"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="7" t="inlineStr">
+      <c r="A1" s="6" t="inlineStr">
         <is>
           <t>DUID</t>
         </is>
       </c>
-      <c r="B1" s="7" t="inlineStr">
+      <c r="B1" s="6" t="inlineStr">
         <is>
           <t>Fuel</t>
         </is>
       </c>
-      <c r="C1" s="7" t="inlineStr">
+      <c r="C1" s="6" t="inlineStr">
         <is>
           <t>MLF_FY25-26</t>
         </is>
       </c>
-      <c r="D1" s="7" t="inlineStr">
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>MLF_FY26-27</t>
         </is>
       </c>
-      <c r="E1" s="7" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>CURTAILMENT_ACTUAL_FY23-24</t>
         </is>
       </c>
-      <c r="F1" s="7" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>CURTAILMENT_ACTUAL_FY24-25</t>
         </is>
       </c>
-      <c r="G1" s="7" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>ELI_CURTAILMENT_NEAR</t>
         </is>
       </c>
-      <c r="H1" s="7" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>ELI_CURTAILMENT_MED</t>
         </is>
       </c>
-      <c r="I1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY1</t>
-        </is>
-      </c>
-      <c r="J1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY1_LABEL</t>
-        </is>
-      </c>
-      <c r="K1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY2</t>
-        </is>
-      </c>
-      <c r="L1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY2_LABEL</t>
-        </is>
-      </c>
-      <c r="M1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY3</t>
-        </is>
-      </c>
-      <c r="N1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_FY3_LABEL</t>
-        </is>
-      </c>
-      <c r="O1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_CURTAILMENT_AVG</t>
-        </is>
-      </c>
-      <c r="P1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY1</t>
-        </is>
-      </c>
-      <c r="Q1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY1_LABEL</t>
-        </is>
-      </c>
-      <c r="R1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY2</t>
-        </is>
-      </c>
-      <c r="S1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY2_LABEL</t>
-        </is>
-      </c>
-      <c r="T1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY3</t>
-        </is>
-      </c>
-      <c r="U1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_FY3_LABEL</t>
-        </is>
-      </c>
-      <c r="V1" s="7" t="inlineStr">
-        <is>
-          <t>ISP_OFFLOADING_AVG</t>
-        </is>
-      </c>
     </row>
     <row r="2">
-      <c r="A2" s="8" t="inlineStr">
+      <c r="A2" s="7" t="inlineStr">
         <is>
           <t>ADPPV1</t>
         </is>
       </c>
-      <c r="B2" s="8" t="inlineStr">
+      <c r="B2" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -3778,52 +3099,14 @@
       </c>
       <c r="G2" s="5" t="inlineStr"/>
       <c r="H2" s="5" t="inlineStr"/>
-      <c r="I2" s="5" t="inlineStr"/>
-      <c r="J2" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr"/>
-      <c r="L2" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M2" s="5" t="inlineStr"/>
-      <c r="N2" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O2" s="5" t="inlineStr"/>
-      <c r="P2" s="5" t="inlineStr"/>
-      <c r="Q2" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R2" s="5" t="inlineStr"/>
-      <c r="S2" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T2" s="5" t="inlineStr"/>
-      <c r="U2" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V2" s="5" t="inlineStr"/>
     </row>
     <row r="3">
-      <c r="A3" s="8" t="inlineStr">
+      <c r="A3" s="7" t="inlineStr">
         <is>
           <t>ADPPV2</t>
         </is>
       </c>
-      <c r="B3" s="8" t="inlineStr">
+      <c r="B3" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -3838,52 +3121,14 @@
       <c r="F3" s="5" t="inlineStr"/>
       <c r="G3" s="5" t="inlineStr"/>
       <c r="H3" s="5" t="inlineStr"/>
-      <c r="I3" s="5" t="inlineStr"/>
-      <c r="J3" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K3" s="5" t="inlineStr"/>
-      <c r="L3" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M3" s="5" t="inlineStr"/>
-      <c r="N3" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O3" s="5" t="inlineStr"/>
-      <c r="P3" s="5" t="inlineStr"/>
-      <c r="Q3" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R3" s="5" t="inlineStr"/>
-      <c r="S3" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T3" s="5" t="inlineStr"/>
-      <c r="U3" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V3" s="5" t="inlineStr"/>
     </row>
     <row r="4">
-      <c r="A4" s="8" t="inlineStr">
+      <c r="A4" s="7" t="inlineStr">
         <is>
           <t>ADPPV3</t>
         </is>
       </c>
-      <c r="B4" s="8" t="inlineStr">
+      <c r="B4" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -3898,52 +3143,14 @@
       <c r="F4" s="5" t="inlineStr"/>
       <c r="G4" s="5" t="inlineStr"/>
       <c r="H4" s="5" t="inlineStr"/>
-      <c r="I4" s="5" t="inlineStr"/>
-      <c r="J4" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K4" s="5" t="inlineStr"/>
-      <c r="L4" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M4" s="5" t="inlineStr"/>
-      <c r="N4" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O4" s="5" t="inlineStr"/>
-      <c r="P4" s="5" t="inlineStr"/>
-      <c r="Q4" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R4" s="5" t="inlineStr"/>
-      <c r="S4" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T4" s="5" t="inlineStr"/>
-      <c r="U4" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V4" s="5" t="inlineStr"/>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>BOWWPV1</t>
         </is>
       </c>
-      <c r="B5" s="8" t="inlineStr">
+      <c r="B5" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -3960,52 +3167,14 @@
       </c>
       <c r="G5" s="5" t="inlineStr"/>
       <c r="H5" s="5" t="inlineStr"/>
-      <c r="I5" s="5" t="inlineStr"/>
-      <c r="J5" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K5" s="5" t="inlineStr"/>
-      <c r="L5" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M5" s="5" t="inlineStr"/>
-      <c r="N5" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O5" s="5" t="inlineStr"/>
-      <c r="P5" s="5" t="inlineStr"/>
-      <c r="Q5" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R5" s="5" t="inlineStr"/>
-      <c r="S5" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T5" s="5" t="inlineStr"/>
-      <c r="U5" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V5" s="5" t="inlineStr"/>
     </row>
     <row r="6">
-      <c r="A6" s="8" t="inlineStr">
+      <c r="A6" s="7" t="inlineStr">
         <is>
           <t>BNGSF1</t>
         </is>
       </c>
-      <c r="B6" s="8" t="inlineStr">
+      <c r="B6" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4028,68 +3197,14 @@
       <c r="H6" s="5" t="n">
         <v>0.212860651220515</v>
       </c>
-      <c r="I6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J6" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L6" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N6" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O6" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P6" s="5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="Q6" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R6" s="5" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="S6" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T6" s="5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="U6" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V6" s="5" t="n">
-        <v>0.07333333333333335</v>
-      </c>
     </row>
     <row r="7">
-      <c r="A7" s="8" t="inlineStr">
+      <c r="A7" s="7" t="inlineStr">
         <is>
           <t>BNGSF2</t>
         </is>
       </c>
-      <c r="B7" s="8" t="inlineStr">
+      <c r="B7" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4112,68 +3227,14 @@
       <c r="H7" s="5" t="n">
         <v>0.212860651220515</v>
       </c>
-      <c r="I7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J7" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L7" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N7" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O7" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P7" s="5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="Q7" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R7" s="5" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="S7" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T7" s="5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="U7" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V7" s="5" t="n">
-        <v>0.07333333333333335</v>
-      </c>
     </row>
     <row r="8">
-      <c r="A8" s="8" t="inlineStr">
+      <c r="A8" s="7" t="inlineStr">
         <is>
           <t>CBWWPV1</t>
         </is>
       </c>
-      <c r="B8" s="8" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4188,52 +3249,14 @@
       <c r="F8" s="5" t="inlineStr"/>
       <c r="G8" s="5" t="inlineStr"/>
       <c r="H8" s="5" t="inlineStr"/>
-      <c r="I8" s="5" t="inlineStr"/>
-      <c r="J8" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K8" s="5" t="inlineStr"/>
-      <c r="L8" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M8" s="5" t="inlineStr"/>
-      <c r="N8" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O8" s="5" t="inlineStr"/>
-      <c r="P8" s="5" t="inlineStr"/>
-      <c r="Q8" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R8" s="5" t="inlineStr"/>
-      <c r="S8" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T8" s="5" t="inlineStr"/>
-      <c r="U8" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V8" s="5" t="inlineStr"/>
     </row>
     <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+      <c r="A9" s="7" t="inlineStr">
         <is>
           <t>CBWWPV2</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B9" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4248,52 +3271,14 @@
       <c r="F9" s="5" t="inlineStr"/>
       <c r="G9" s="5" t="inlineStr"/>
       <c r="H9" s="5" t="inlineStr"/>
-      <c r="I9" s="5" t="inlineStr"/>
-      <c r="J9" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K9" s="5" t="inlineStr"/>
-      <c r="L9" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M9" s="5" t="inlineStr"/>
-      <c r="N9" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O9" s="5" t="inlineStr"/>
-      <c r="P9" s="5" t="inlineStr"/>
-      <c r="Q9" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R9" s="5" t="inlineStr"/>
-      <c r="S9" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T9" s="5" t="inlineStr"/>
-      <c r="U9" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V9" s="5" t="inlineStr"/>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
+      <c r="A10" s="7" t="inlineStr">
         <is>
           <t>HVWWPV1</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B10" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4316,52 +3301,14 @@
       <c r="H10" s="5" t="n">
         <v>0.22265637813532</v>
       </c>
-      <c r="I10" s="5" t="inlineStr"/>
-      <c r="J10" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K10" s="5" t="inlineStr"/>
-      <c r="L10" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M10" s="5" t="inlineStr"/>
-      <c r="N10" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O10" s="5" t="inlineStr"/>
-      <c r="P10" s="5" t="inlineStr"/>
-      <c r="Q10" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R10" s="5" t="inlineStr"/>
-      <c r="S10" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T10" s="5" t="inlineStr"/>
-      <c r="U10" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V10" s="5" t="inlineStr"/>
     </row>
     <row r="11">
-      <c r="A11" s="8" t="inlineStr">
+      <c r="A11" s="7" t="inlineStr">
         <is>
           <t>MAPS2PV1</t>
         </is>
       </c>
-      <c r="B11" s="8" t="inlineStr">
+      <c r="B11" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4384,68 +3331,14 @@
       <c r="H11" s="5" t="n">
         <v>0.225784053085401</v>
       </c>
-      <c r="I11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J11" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L11" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N11" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q11" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S11" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T11" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U11" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V11" s="5" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="12">
-      <c r="A12" s="8" t="inlineStr">
+      <c r="A12" s="7" t="inlineStr">
         <is>
           <t>MAPS3PV1</t>
         </is>
       </c>
-      <c r="B12" s="8" t="inlineStr">
+      <c r="B12" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4466,68 +3359,14 @@
       <c r="H12" s="5" t="n">
         <v>0.225784053085401</v>
       </c>
-      <c r="I12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L12" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N12" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q12" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S12" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T12" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U12" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V12" s="5" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="13">
-      <c r="A13" s="8" t="inlineStr">
+      <c r="A13" s="7" t="inlineStr">
         <is>
           <t>MANNSF2</t>
         </is>
       </c>
-      <c r="B13" s="8" t="inlineStr">
+      <c r="B13" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4548,68 +3387,14 @@
       <c r="H13" s="5" t="n">
         <v>0.225784053085401</v>
       </c>
-      <c r="I13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J13" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L13" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N13" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O13" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P13" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="Q13" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R13" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="S13" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T13" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U13" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V13" s="5" t="n">
-        <v>0.16</v>
-      </c>
     </row>
     <row r="14">
-      <c r="A14" s="8" t="inlineStr">
+      <c r="A14" s="7" t="inlineStr">
         <is>
           <t>MWPS1PV1</t>
         </is>
       </c>
-      <c r="B14" s="8" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4632,68 +3417,14 @@
       <c r="H14" s="5" t="n">
         <v>0.512670422089759</v>
       </c>
-      <c r="I14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J14" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L14" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N14" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O14" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P14" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="Q14" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R14" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="S14" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T14" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U14" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V14" s="5" t="n">
-        <v>0.16</v>
-      </c>
     </row>
     <row r="15">
-      <c r="A15" s="8" t="inlineStr">
+      <c r="A15" s="7" t="inlineStr">
         <is>
           <t>MWPS2PV1</t>
         </is>
       </c>
-      <c r="B15" s="8" t="inlineStr">
+      <c r="B15" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4716,68 +3447,14 @@
       <c r="H15" s="5" t="n">
         <v>0.512670422089759</v>
       </c>
-      <c r="I15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J15" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L15" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N15" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O15" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P15" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="Q15" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R15" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="S15" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T15" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U15" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V15" s="5" t="n">
-        <v>0.16</v>
-      </c>
     </row>
     <row r="16">
-      <c r="A16" s="8" t="inlineStr">
+      <c r="A16" s="7" t="inlineStr">
         <is>
           <t>MWPS3PV1</t>
         </is>
       </c>
-      <c r="B16" s="8" t="inlineStr">
+      <c r="B16" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4800,68 +3477,14 @@
       <c r="H16" s="5" t="n">
         <v>0.512670422089759</v>
       </c>
-      <c r="I16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J16" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L16" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N16" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O16" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P16" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="Q16" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R16" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="S16" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T16" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U16" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V16" s="5" t="n">
-        <v>0.16</v>
-      </c>
     </row>
     <row r="17">
-      <c r="A17" s="8" t="inlineStr">
+      <c r="A17" s="7" t="inlineStr">
         <is>
           <t>MWPS4PV1</t>
         </is>
       </c>
-      <c r="B17" s="8" t="inlineStr">
+      <c r="B17" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4884,68 +3507,14 @@
       <c r="H17" s="5" t="n">
         <v>0.512670422089759</v>
       </c>
-      <c r="I17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J17" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L17" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N17" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O17" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P17" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="Q17" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R17" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="S17" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T17" s="5" t="n">
-        <v>0.16</v>
-      </c>
-      <c r="U17" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V17" s="5" t="n">
-        <v>0.16</v>
-      </c>
     </row>
     <row r="18">
-      <c r="A18" s="8" t="inlineStr">
+      <c r="A18" s="7" t="inlineStr">
         <is>
           <t>MBPS2PV1</t>
         </is>
       </c>
-      <c r="B18" s="8" t="inlineStr">
+      <c r="B18" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -4968,68 +3537,14 @@
       <c r="H18" s="5" t="n">
         <v>0.225784053085401</v>
       </c>
-      <c r="I18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J18" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L18" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N18" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q18" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S18" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T18" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="U18" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V18" s="5" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="19">
-      <c r="A19" s="8" t="inlineStr">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>PAREPS1</t>
         </is>
       </c>
-      <c r="B19" s="8" t="inlineStr">
+      <c r="B19" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -5052,68 +3567,14 @@
       <c r="H19" s="5" t="n">
         <v>0.212860651220515</v>
       </c>
-      <c r="I19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J19" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L19" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="N19" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O19" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P19" s="5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="Q19" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R19" s="5" t="n">
-        <v>0.08</v>
-      </c>
-      <c r="S19" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T19" s="5" t="n">
-        <v>0.07000000000000001</v>
-      </c>
-      <c r="U19" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V19" s="5" t="n">
-        <v>0.07333333333333335</v>
-      </c>
     </row>
     <row r="20">
-      <c r="A20" s="8" t="inlineStr">
+      <c r="A20" s="7" t="inlineStr">
         <is>
           <t>TB2SF1</t>
         </is>
       </c>
-      <c r="B20" s="8" t="inlineStr">
+      <c r="B20" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -5136,52 +3597,14 @@
       <c r="H20" s="5" t="n">
         <v>0.22945882760626</v>
       </c>
-      <c r="I20" s="5" t="inlineStr"/>
-      <c r="J20" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K20" s="5" t="inlineStr"/>
-      <c r="L20" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M20" s="5" t="inlineStr"/>
-      <c r="N20" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O20" s="5" t="inlineStr"/>
-      <c r="P20" s="5" t="inlineStr"/>
-      <c r="Q20" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R20" s="5" t="inlineStr"/>
-      <c r="S20" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T20" s="5" t="inlineStr"/>
-      <c r="U20" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V20" s="5" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="8" t="inlineStr">
+      <c r="A21" s="7" t="inlineStr">
         <is>
           <t>TBSF1</t>
         </is>
       </c>
-      <c r="B21" s="8" t="inlineStr">
+      <c r="B21" s="7" t="inlineStr">
         <is>
           <t>Solar</t>
         </is>
@@ -5204,52 +3627,14 @@
       <c r="H21" s="5" t="n">
         <v>0.22945882760626</v>
       </c>
-      <c r="I21" s="5" t="inlineStr"/>
-      <c r="J21" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K21" s="5" t="inlineStr"/>
-      <c r="L21" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M21" s="5" t="inlineStr"/>
-      <c r="N21" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O21" s="5" t="inlineStr"/>
-      <c r="P21" s="5" t="inlineStr"/>
-      <c r="Q21" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R21" s="5" t="inlineStr"/>
-      <c r="S21" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T21" s="5" t="inlineStr"/>
-      <c r="U21" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V21" s="5" t="inlineStr"/>
     </row>
     <row r="22">
-      <c r="A22" s="8" t="inlineStr">
+      <c r="A22" s="7" t="inlineStr">
         <is>
           <t>CNUNDAWF</t>
         </is>
       </c>
-      <c r="B22" s="8" t="inlineStr">
+      <c r="B22" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5268,52 +3653,14 @@
       </c>
       <c r="G22" s="5" t="inlineStr"/>
       <c r="H22" s="5" t="inlineStr"/>
-      <c r="I22" s="5" t="inlineStr"/>
-      <c r="J22" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K22" s="5" t="inlineStr"/>
-      <c r="L22" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M22" s="5" t="inlineStr"/>
-      <c r="N22" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O22" s="5" t="inlineStr"/>
-      <c r="P22" s="5" t="inlineStr"/>
-      <c r="Q22" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R22" s="5" t="inlineStr"/>
-      <c r="S22" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T22" s="5" t="inlineStr"/>
-      <c r="U22" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V22" s="5" t="inlineStr"/>
     </row>
     <row r="23">
-      <c r="A23" s="8" t="inlineStr">
+      <c r="A23" s="7" t="inlineStr">
         <is>
           <t>CATHROCK</t>
         </is>
       </c>
-      <c r="B23" s="8" t="inlineStr">
+      <c r="B23" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5332,52 +3679,14 @@
       </c>
       <c r="G23" s="5" t="inlineStr"/>
       <c r="H23" s="5" t="inlineStr"/>
-      <c r="I23" s="5" t="inlineStr"/>
-      <c r="J23" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K23" s="5" t="inlineStr"/>
-      <c r="L23" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M23" s="5" t="inlineStr"/>
-      <c r="N23" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O23" s="5" t="inlineStr"/>
-      <c r="P23" s="5" t="inlineStr"/>
-      <c r="Q23" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R23" s="5" t="inlineStr"/>
-      <c r="S23" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T23" s="5" t="inlineStr"/>
-      <c r="U23" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V23" s="5" t="inlineStr"/>
     </row>
     <row r="24">
-      <c r="A24" s="8" t="inlineStr">
+      <c r="A24" s="7" t="inlineStr">
         <is>
           <t>CLEMGPWF</t>
         </is>
       </c>
-      <c r="B24" s="8" t="inlineStr">
+      <c r="B24" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5396,52 +3705,14 @@
       </c>
       <c r="G24" s="5" t="inlineStr"/>
       <c r="H24" s="5" t="inlineStr"/>
-      <c r="I24" s="5" t="inlineStr"/>
-      <c r="J24" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K24" s="5" t="inlineStr"/>
-      <c r="L24" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M24" s="5" t="inlineStr"/>
-      <c r="N24" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O24" s="5" t="inlineStr"/>
-      <c r="P24" s="5" t="inlineStr"/>
-      <c r="Q24" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R24" s="5" t="inlineStr"/>
-      <c r="S24" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T24" s="5" t="inlineStr"/>
-      <c r="U24" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V24" s="5" t="inlineStr"/>
     </row>
     <row r="25">
-      <c r="A25" s="8" t="inlineStr">
+      <c r="A25" s="7" t="inlineStr">
         <is>
           <t>GSWF1A</t>
         </is>
       </c>
-      <c r="B25" s="8" t="inlineStr">
+      <c r="B25" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5458,52 +3729,14 @@
       </c>
       <c r="G25" s="5" t="inlineStr"/>
       <c r="H25" s="5" t="inlineStr"/>
-      <c r="I25" s="5" t="inlineStr"/>
-      <c r="J25" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K25" s="5" t="inlineStr"/>
-      <c r="L25" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M25" s="5" t="inlineStr"/>
-      <c r="N25" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O25" s="5" t="inlineStr"/>
-      <c r="P25" s="5" t="inlineStr"/>
-      <c r="Q25" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R25" s="5" t="inlineStr"/>
-      <c r="S25" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T25" s="5" t="inlineStr"/>
-      <c r="U25" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V25" s="5" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="8" t="inlineStr">
+      <c r="A26" s="7" t="inlineStr">
         <is>
           <t>GSWF1B1</t>
         </is>
       </c>
-      <c r="B26" s="8" t="inlineStr">
+      <c r="B26" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5518,52 +3751,14 @@
       <c r="F26" s="5" t="inlineStr"/>
       <c r="G26" s="5" t="inlineStr"/>
       <c r="H26" s="5" t="inlineStr"/>
-      <c r="I26" s="5" t="inlineStr"/>
-      <c r="J26" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K26" s="5" t="inlineStr"/>
-      <c r="L26" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M26" s="5" t="inlineStr"/>
-      <c r="N26" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O26" s="5" t="inlineStr"/>
-      <c r="P26" s="5" t="inlineStr"/>
-      <c r="Q26" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R26" s="5" t="inlineStr"/>
-      <c r="S26" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T26" s="5" t="inlineStr"/>
-      <c r="U26" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V26" s="5" t="inlineStr"/>
     </row>
     <row r="27">
-      <c r="A27" s="8" t="inlineStr">
+      <c r="A27" s="7" t="inlineStr">
         <is>
           <t>HALLWF1</t>
         </is>
       </c>
-      <c r="B27" s="8" t="inlineStr">
+      <c r="B27" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5582,52 +3777,14 @@
       </c>
       <c r="G27" s="5" t="inlineStr"/>
       <c r="H27" s="5" t="inlineStr"/>
-      <c r="I27" s="5" t="inlineStr"/>
-      <c r="J27" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K27" s="5" t="inlineStr"/>
-      <c r="L27" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M27" s="5" t="inlineStr"/>
-      <c r="N27" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O27" s="5" t="inlineStr"/>
-      <c r="P27" s="5" t="inlineStr"/>
-      <c r="Q27" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R27" s="5" t="inlineStr"/>
-      <c r="S27" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T27" s="5" t="inlineStr"/>
-      <c r="U27" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V27" s="5" t="inlineStr"/>
     </row>
     <row r="28">
-      <c r="A28" s="8" t="inlineStr">
+      <c r="A28" s="7" t="inlineStr">
         <is>
           <t>HALLWF2</t>
         </is>
       </c>
-      <c r="B28" s="8" t="inlineStr">
+      <c r="B28" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5646,52 +3803,14 @@
       </c>
       <c r="G28" s="5" t="inlineStr"/>
       <c r="H28" s="5" t="inlineStr"/>
-      <c r="I28" s="5" t="inlineStr"/>
-      <c r="J28" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K28" s="5" t="inlineStr"/>
-      <c r="L28" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M28" s="5" t="inlineStr"/>
-      <c r="N28" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O28" s="5" t="inlineStr"/>
-      <c r="P28" s="5" t="inlineStr"/>
-      <c r="Q28" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R28" s="5" t="inlineStr"/>
-      <c r="S28" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T28" s="5" t="inlineStr"/>
-      <c r="U28" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V28" s="5" t="inlineStr"/>
     </row>
     <row r="29">
-      <c r="A29" s="8" t="inlineStr">
+      <c r="A29" s="7" t="inlineStr">
         <is>
           <t>HDWF1</t>
         </is>
       </c>
-      <c r="B29" s="8" t="inlineStr">
+      <c r="B29" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5710,52 +3829,14 @@
       </c>
       <c r="G29" s="5" t="inlineStr"/>
       <c r="H29" s="5" t="inlineStr"/>
-      <c r="I29" s="5" t="inlineStr"/>
-      <c r="J29" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K29" s="5" t="inlineStr"/>
-      <c r="L29" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M29" s="5" t="inlineStr"/>
-      <c r="N29" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O29" s="5" t="inlineStr"/>
-      <c r="P29" s="5" t="inlineStr"/>
-      <c r="Q29" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R29" s="5" t="inlineStr"/>
-      <c r="S29" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T29" s="5" t="inlineStr"/>
-      <c r="U29" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V29" s="5" t="inlineStr"/>
     </row>
     <row r="30">
-      <c r="A30" s="8" t="inlineStr">
+      <c r="A30" s="7" t="inlineStr">
         <is>
           <t>HDWF2</t>
         </is>
       </c>
-      <c r="B30" s="8" t="inlineStr">
+      <c r="B30" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5774,52 +3855,14 @@
       </c>
       <c r="G30" s="5" t="inlineStr"/>
       <c r="H30" s="5" t="inlineStr"/>
-      <c r="I30" s="5" t="inlineStr"/>
-      <c r="J30" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K30" s="5" t="inlineStr"/>
-      <c r="L30" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M30" s="5" t="inlineStr"/>
-      <c r="N30" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O30" s="5" t="inlineStr"/>
-      <c r="P30" s="5" t="inlineStr"/>
-      <c r="Q30" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R30" s="5" t="inlineStr"/>
-      <c r="S30" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T30" s="5" t="inlineStr"/>
-      <c r="U30" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V30" s="5" t="inlineStr"/>
     </row>
     <row r="31">
-      <c r="A31" s="8" t="inlineStr">
+      <c r="A31" s="7" t="inlineStr">
         <is>
           <t>HDWF3</t>
         </is>
       </c>
-      <c r="B31" s="8" t="inlineStr">
+      <c r="B31" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5838,52 +3881,14 @@
       </c>
       <c r="G31" s="5" t="inlineStr"/>
       <c r="H31" s="5" t="inlineStr"/>
-      <c r="I31" s="5" t="inlineStr"/>
-      <c r="J31" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K31" s="5" t="inlineStr"/>
-      <c r="L31" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M31" s="5" t="inlineStr"/>
-      <c r="N31" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O31" s="5" t="inlineStr"/>
-      <c r="P31" s="5" t="inlineStr"/>
-      <c r="Q31" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R31" s="5" t="inlineStr"/>
-      <c r="S31" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T31" s="5" t="inlineStr"/>
-      <c r="U31" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V31" s="5" t="inlineStr"/>
     </row>
     <row r="32">
-      <c r="A32" s="8" t="inlineStr">
+      <c r="A32" s="7" t="inlineStr">
         <is>
           <t>LKBONNY2</t>
         </is>
       </c>
-      <c r="B32" s="8" t="inlineStr">
+      <c r="B32" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5902,52 +3907,14 @@
       </c>
       <c r="G32" s="5" t="inlineStr"/>
       <c r="H32" s="5" t="inlineStr"/>
-      <c r="I32" s="5" t="inlineStr"/>
-      <c r="J32" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K32" s="5" t="inlineStr"/>
-      <c r="L32" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M32" s="5" t="inlineStr"/>
-      <c r="N32" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O32" s="5" t="inlineStr"/>
-      <c r="P32" s="5" t="inlineStr"/>
-      <c r="Q32" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R32" s="5" t="inlineStr"/>
-      <c r="S32" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T32" s="5" t="inlineStr"/>
-      <c r="U32" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V32" s="5" t="inlineStr"/>
     </row>
     <row r="33">
-      <c r="A33" s="8" t="inlineStr">
+      <c r="A33" s="7" t="inlineStr">
         <is>
           <t>LKBONNY3</t>
         </is>
       </c>
-      <c r="B33" s="8" t="inlineStr">
+      <c r="B33" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -5966,52 +3933,14 @@
       </c>
       <c r="G33" s="5" t="inlineStr"/>
       <c r="H33" s="5" t="inlineStr"/>
-      <c r="I33" s="5" t="inlineStr"/>
-      <c r="J33" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K33" s="5" t="inlineStr"/>
-      <c r="L33" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M33" s="5" t="inlineStr"/>
-      <c r="N33" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O33" s="5" t="inlineStr"/>
-      <c r="P33" s="5" t="inlineStr"/>
-      <c r="Q33" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R33" s="5" t="inlineStr"/>
-      <c r="S33" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T33" s="5" t="inlineStr"/>
-      <c r="U33" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V33" s="5" t="inlineStr"/>
     </row>
     <row r="34">
-      <c r="A34" s="8" t="inlineStr">
+      <c r="A34" s="7" t="inlineStr">
         <is>
           <t>LKBONNY1</t>
         </is>
       </c>
-      <c r="B34" s="8" t="inlineStr">
+      <c r="B34" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6030,52 +3959,14 @@
       </c>
       <c r="G34" s="5" t="inlineStr"/>
       <c r="H34" s="5" t="inlineStr"/>
-      <c r="I34" s="5" t="inlineStr"/>
-      <c r="J34" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K34" s="5" t="inlineStr"/>
-      <c r="L34" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M34" s="5" t="inlineStr"/>
-      <c r="N34" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O34" s="5" t="inlineStr"/>
-      <c r="P34" s="5" t="inlineStr"/>
-      <c r="Q34" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R34" s="5" t="inlineStr"/>
-      <c r="S34" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T34" s="5" t="inlineStr"/>
-      <c r="U34" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V34" s="5" t="inlineStr"/>
     </row>
     <row r="35">
-      <c r="A35" s="8" t="inlineStr">
+      <c r="A35" s="7" t="inlineStr">
         <is>
           <t>LGAPWF1</t>
         </is>
       </c>
-      <c r="B35" s="8" t="inlineStr">
+      <c r="B35" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6094,52 +3985,14 @@
       </c>
       <c r="G35" s="5" t="inlineStr"/>
       <c r="H35" s="5" t="inlineStr"/>
-      <c r="I35" s="5" t="inlineStr"/>
-      <c r="J35" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K35" s="5" t="inlineStr"/>
-      <c r="L35" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M35" s="5" t="inlineStr"/>
-      <c r="N35" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O35" s="5" t="inlineStr"/>
-      <c r="P35" s="5" t="inlineStr"/>
-      <c r="Q35" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R35" s="5" t="inlineStr"/>
-      <c r="S35" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T35" s="5" t="inlineStr"/>
-      <c r="U35" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V35" s="5" t="inlineStr"/>
     </row>
     <row r="36">
-      <c r="A36" s="8" t="inlineStr">
+      <c r="A36" s="7" t="inlineStr">
         <is>
           <t>LGAPWF2</t>
         </is>
       </c>
-      <c r="B36" s="8" t="inlineStr">
+      <c r="B36" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6158,52 +4011,14 @@
       </c>
       <c r="G36" s="5" t="inlineStr"/>
       <c r="H36" s="5" t="inlineStr"/>
-      <c r="I36" s="5" t="inlineStr"/>
-      <c r="J36" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K36" s="5" t="inlineStr"/>
-      <c r="L36" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M36" s="5" t="inlineStr"/>
-      <c r="N36" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O36" s="5" t="inlineStr"/>
-      <c r="P36" s="5" t="inlineStr"/>
-      <c r="Q36" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R36" s="5" t="inlineStr"/>
-      <c r="S36" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T36" s="5" t="inlineStr"/>
-      <c r="U36" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V36" s="5" t="inlineStr"/>
     </row>
     <row r="37">
-      <c r="A37" s="8" t="inlineStr">
+      <c r="A37" s="7" t="inlineStr">
         <is>
           <t>MTMILLAR</t>
         </is>
       </c>
-      <c r="B37" s="8" t="inlineStr">
+      <c r="B37" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6222,52 +4037,14 @@
       </c>
       <c r="G37" s="5" t="inlineStr"/>
       <c r="H37" s="5" t="inlineStr"/>
-      <c r="I37" s="5" t="inlineStr"/>
-      <c r="J37" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K37" s="5" t="inlineStr"/>
-      <c r="L37" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M37" s="5" t="inlineStr"/>
-      <c r="N37" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O37" s="5" t="inlineStr"/>
-      <c r="P37" s="5" t="inlineStr"/>
-      <c r="Q37" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R37" s="5" t="inlineStr"/>
-      <c r="S37" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T37" s="5" t="inlineStr"/>
-      <c r="U37" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V37" s="5" t="inlineStr"/>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>NBHWF1</t>
         </is>
       </c>
-      <c r="B38" s="8" t="inlineStr">
+      <c r="B38" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6286,52 +4063,14 @@
       </c>
       <c r="G38" s="5" t="inlineStr"/>
       <c r="H38" s="5" t="inlineStr"/>
-      <c r="I38" s="5" t="inlineStr"/>
-      <c r="J38" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K38" s="5" t="inlineStr"/>
-      <c r="L38" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M38" s="5" t="inlineStr"/>
-      <c r="N38" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O38" s="5" t="inlineStr"/>
-      <c r="P38" s="5" t="inlineStr"/>
-      <c r="Q38" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R38" s="5" t="inlineStr"/>
-      <c r="S38" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T38" s="5" t="inlineStr"/>
-      <c r="U38" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V38" s="5" t="inlineStr"/>
     </row>
     <row r="39">
-      <c r="A39" s="8" t="inlineStr">
+      <c r="A39" s="7" t="inlineStr">
         <is>
           <t>PAREPW1</t>
         </is>
       </c>
-      <c r="B39" s="8" t="inlineStr">
+      <c r="B39" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6350,52 +4089,14 @@
       </c>
       <c r="G39" s="5" t="inlineStr"/>
       <c r="H39" s="5" t="inlineStr"/>
-      <c r="I39" s="5" t="inlineStr"/>
-      <c r="J39" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K39" s="5" t="inlineStr"/>
-      <c r="L39" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M39" s="5" t="inlineStr"/>
-      <c r="N39" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O39" s="5" t="inlineStr"/>
-      <c r="P39" s="5" t="inlineStr"/>
-      <c r="Q39" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R39" s="5" t="inlineStr"/>
-      <c r="S39" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T39" s="5" t="inlineStr"/>
-      <c r="U39" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V39" s="5" t="inlineStr"/>
     </row>
     <row r="40">
-      <c r="A40" s="8" t="inlineStr">
+      <c r="A40" s="7" t="inlineStr">
         <is>
           <t>SNOWSTH1</t>
         </is>
       </c>
-      <c r="B40" s="8" t="inlineStr">
+      <c r="B40" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6414,52 +4115,14 @@
       </c>
       <c r="G40" s="5" t="inlineStr"/>
       <c r="H40" s="5" t="inlineStr"/>
-      <c r="I40" s="5" t="inlineStr"/>
-      <c r="J40" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K40" s="5" t="inlineStr"/>
-      <c r="L40" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M40" s="5" t="inlineStr"/>
-      <c r="N40" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O40" s="5" t="inlineStr"/>
-      <c r="P40" s="5" t="inlineStr"/>
-      <c r="Q40" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R40" s="5" t="inlineStr"/>
-      <c r="S40" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T40" s="5" t="inlineStr"/>
-      <c r="U40" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V40" s="5" t="inlineStr"/>
     </row>
     <row r="41">
-      <c r="A41" s="8" t="inlineStr">
+      <c r="A41" s="7" t="inlineStr">
         <is>
           <t>SNOWNTH1</t>
         </is>
       </c>
-      <c r="B41" s="8" t="inlineStr">
+      <c r="B41" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6478,52 +4141,14 @@
       </c>
       <c r="G41" s="5" t="inlineStr"/>
       <c r="H41" s="5" t="inlineStr"/>
-      <c r="I41" s="5" t="inlineStr"/>
-      <c r="J41" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K41" s="5" t="inlineStr"/>
-      <c r="L41" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M41" s="5" t="inlineStr"/>
-      <c r="N41" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O41" s="5" t="inlineStr"/>
-      <c r="P41" s="5" t="inlineStr"/>
-      <c r="Q41" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R41" s="5" t="inlineStr"/>
-      <c r="S41" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T41" s="5" t="inlineStr"/>
-      <c r="U41" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V41" s="5" t="inlineStr"/>
     </row>
     <row r="42">
-      <c r="A42" s="8" t="inlineStr">
+      <c r="A42" s="7" t="inlineStr">
         <is>
           <t>SNOWTWN1</t>
         </is>
       </c>
-      <c r="B42" s="8" t="inlineStr">
+      <c r="B42" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6542,52 +4167,14 @@
       </c>
       <c r="G42" s="5" t="inlineStr"/>
       <c r="H42" s="5" t="inlineStr"/>
-      <c r="I42" s="5" t="inlineStr"/>
-      <c r="J42" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K42" s="5" t="inlineStr"/>
-      <c r="L42" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M42" s="5" t="inlineStr"/>
-      <c r="N42" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O42" s="5" t="inlineStr"/>
-      <c r="P42" s="5" t="inlineStr"/>
-      <c r="Q42" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R42" s="5" t="inlineStr"/>
-      <c r="S42" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T42" s="5" t="inlineStr"/>
-      <c r="U42" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V42" s="5" t="inlineStr"/>
     </row>
     <row r="43">
-      <c r="A43" s="8" t="inlineStr">
+      <c r="A43" s="7" t="inlineStr">
         <is>
           <t>STARHLWF</t>
         </is>
       </c>
-      <c r="B43" s="8" t="inlineStr">
+      <c r="B43" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6606,52 +4193,14 @@
       </c>
       <c r="G43" s="5" t="inlineStr"/>
       <c r="H43" s="5" t="inlineStr"/>
-      <c r="I43" s="5" t="inlineStr"/>
-      <c r="J43" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K43" s="5" t="inlineStr"/>
-      <c r="L43" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M43" s="5" t="inlineStr"/>
-      <c r="N43" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O43" s="5" t="inlineStr"/>
-      <c r="P43" s="5" t="inlineStr"/>
-      <c r="Q43" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R43" s="5" t="inlineStr"/>
-      <c r="S43" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T43" s="5" t="inlineStr"/>
-      <c r="U43" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V43" s="5" t="inlineStr"/>
     </row>
     <row r="44">
-      <c r="A44" s="8" t="inlineStr">
+      <c r="A44" s="7" t="inlineStr">
         <is>
           <t>BLUFF1</t>
         </is>
       </c>
-      <c r="B44" s="8" t="inlineStr">
+      <c r="B44" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6670,52 +4219,14 @@
       </c>
       <c r="G44" s="5" t="inlineStr"/>
       <c r="H44" s="5" t="inlineStr"/>
-      <c r="I44" s="5" t="inlineStr"/>
-      <c r="J44" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K44" s="5" t="inlineStr"/>
-      <c r="L44" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M44" s="5" t="inlineStr"/>
-      <c r="N44" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O44" s="5" t="inlineStr"/>
-      <c r="P44" s="5" t="inlineStr"/>
-      <c r="Q44" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R44" s="5" t="inlineStr"/>
-      <c r="S44" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T44" s="5" t="inlineStr"/>
-      <c r="U44" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V44" s="5" t="inlineStr"/>
     </row>
     <row r="45">
-      <c r="A45" s="8" t="inlineStr">
+      <c r="A45" s="7" t="inlineStr">
         <is>
           <t>WATERLWF</t>
         </is>
       </c>
-      <c r="B45" s="8" t="inlineStr">
+      <c r="B45" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6734,52 +4245,14 @@
       </c>
       <c r="G45" s="5" t="inlineStr"/>
       <c r="H45" s="5" t="inlineStr"/>
-      <c r="I45" s="5" t="inlineStr"/>
-      <c r="J45" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K45" s="5" t="inlineStr"/>
-      <c r="L45" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M45" s="5" t="inlineStr"/>
-      <c r="N45" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O45" s="5" t="inlineStr"/>
-      <c r="P45" s="5" t="inlineStr"/>
-      <c r="Q45" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R45" s="5" t="inlineStr"/>
-      <c r="S45" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T45" s="5" t="inlineStr"/>
-      <c r="U45" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V45" s="5" t="inlineStr"/>
     </row>
     <row r="46">
-      <c r="A46" s="8" t="inlineStr">
+      <c r="A46" s="7" t="inlineStr">
         <is>
           <t>WPWF</t>
         </is>
       </c>
-      <c r="B46" s="8" t="inlineStr">
+      <c r="B46" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6798,52 +4271,14 @@
       </c>
       <c r="G46" s="5" t="inlineStr"/>
       <c r="H46" s="5" t="inlineStr"/>
-      <c r="I46" s="5" t="inlineStr"/>
-      <c r="J46" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K46" s="5" t="inlineStr"/>
-      <c r="L46" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M46" s="5" t="inlineStr"/>
-      <c r="N46" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O46" s="5" t="inlineStr"/>
-      <c r="P46" s="5" t="inlineStr"/>
-      <c r="Q46" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R46" s="5" t="inlineStr"/>
-      <c r="S46" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T46" s="5" t="inlineStr"/>
-      <c r="U46" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V46" s="5" t="inlineStr"/>
     </row>
     <row r="47">
-      <c r="A47" s="8" t="inlineStr">
+      <c r="A47" s="7" t="inlineStr">
         <is>
           <t>WGWF1</t>
         </is>
       </c>
-      <c r="B47" s="8" t="inlineStr">
+      <c r="B47" s="7" t="inlineStr">
         <is>
           <t>Wind</t>
         </is>
@@ -6862,44 +4297,6 @@
       </c>
       <c r="G47" s="5" t="inlineStr"/>
       <c r="H47" s="5" t="inlineStr"/>
-      <c r="I47" s="5" t="inlineStr"/>
-      <c r="J47" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="K47" s="5" t="inlineStr"/>
-      <c r="L47" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="M47" s="5" t="inlineStr"/>
-      <c r="N47" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="O47" s="5" t="inlineStr"/>
-      <c r="P47" s="5" t="inlineStr"/>
-      <c r="Q47" s="5" t="inlineStr">
-        <is>
-          <t>25-26</t>
-        </is>
-      </c>
-      <c r="R47" s="5" t="inlineStr"/>
-      <c r="S47" s="5" t="inlineStr">
-        <is>
-          <t>26-27</t>
-        </is>
-      </c>
-      <c r="T47" s="5" t="inlineStr"/>
-      <c r="U47" s="5" t="inlineStr">
-        <is>
-          <t>27-28</t>
-        </is>
-      </c>
-      <c r="V47" s="5" t="inlineStr"/>
     </row>
   </sheetData>
   <conditionalFormatting sqref="C2:C47">
@@ -6974,174 +4371,6 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="I2:I47">
-    <cfRule type="colorScale" priority="7">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="J2:J47">
-    <cfRule type="colorScale" priority="8">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="K2:K47">
-    <cfRule type="colorScale" priority="9">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="L2:L47">
-    <cfRule type="colorScale" priority="10">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="M2:M47">
-    <cfRule type="colorScale" priority="11">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="N2:N47">
-    <cfRule type="colorScale" priority="12">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="O2:O47">
-    <cfRule type="colorScale" priority="13">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="P2:P47">
-    <cfRule type="colorScale" priority="14">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="Q2:Q47">
-    <cfRule type="colorScale" priority="15">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="R2:R47">
-    <cfRule type="colorScale" priority="16">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="S2:S47">
-    <cfRule type="colorScale" priority="17">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="T2:T47">
-    <cfRule type="colorScale" priority="18">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="U2:U47">
-    <cfRule type="colorScale" priority="19">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="V2:V47">
-    <cfRule type="colorScale" priority="20">
-      <colorScale>
-        <cfvo type="min"/>
-        <cfvo type="percentile" val="50"/>
-        <cfvo type="max"/>
-        <color rgb="0063BE7B"/>
-        <color rgb="00FFEB84"/>
-        <color rgb="00F8696B"/>
-      </colorScale>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>